<commit_message>
Plan de trabajo y lecturas de la mentoría
</commit_message>
<xml_diff>
--- a/Mentoria_Fernando.xlsx
+++ b/Mentoria_Fernando.xlsx
@@ -8,14 +8,16 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi cabina" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi preparación" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi Radar IA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis metas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis compromisos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis avances" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acuerdo" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas de metas" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_info" sheetId="9" state="veryHidden" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis lecturas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi preparación" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi Radar IA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis metas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis compromisos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mis avances" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acuerdo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas de metas" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_info" sheetId="11" state="veryHidden" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +64,12 @@
       <name val="Calibri"/>
       <color rgb="000A1A3F"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002563EB"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -261,44 +269,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -307,13 +315,13 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -322,10 +330,10 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -334,15 +342,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -466,7 +477,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblFPreparacion" displayName="tblFPreparacion" ref="A4:B9" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblFPlan" displayName="tblFPlan" ref="A4:D10" headerRowCount="1">
+  <autoFilter ref="A4:D10"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Sesión"/>
+    <tableColumn id="2" name="Enfoque"/>
+    <tableColumn id="3" name="Lo que me toca"/>
+    <tableColumn id="4" name="Entregable"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblFSugeridas" displayName="tblFSugeridas" ref="A4:D11" headerRowCount="1">
+  <autoFilter ref="A4:D11"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Meta"/>
+    <tableColumn id="2" name="M · Medible"/>
+    <tableColumn id="3" name="Plazo (días)"/>
+    <tableColumn id="4" name="Área"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblFInfo" displayName="tblFInfo" ref="A1:B5" headerRowCount="1">
+  <autoFilter ref="A1:B5"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Clave"/>
+    <tableColumn id="2" name="Valor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblFLecturas" displayName="tblFLecturas" ref="A4:G11" headerRowCount="1">
+  <autoFilter ref="A4:G11"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Sesión"/>
+    <tableColumn id="2" name="Título"/>
+    <tableColumn id="3" name="Autor"/>
+    <tableColumn id="4" name="Formato"/>
+    <tableColumn id="5" name="Minutos"/>
+    <tableColumn id="6" name="Por qué leerla"/>
+    <tableColumn id="7" name="Liga"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblFPreparacion" displayName="tblFPreparacion" ref="A4:B9" headerRowCount="1">
   <autoFilter ref="A4:B9"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Tarea"/>
@@ -476,8 +540,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblFRadar" displayName="tblFRadar" ref="A4:E11" headerRowCount="1">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblFRadar" displayName="tblFRadar" ref="A4:E11" headerRowCount="1">
   <autoFilter ref="A4:E11"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Área"/>
@@ -490,8 +554,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblFNiveles" displayName="tblFNiveles" ref="A15:C20" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblFNiveles" displayName="tblFNiveles" ref="A15:C20" headerRowCount="1">
   <autoFilter ref="A15:C20"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Nombre"/>
@@ -502,8 +566,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblFMetas" displayName="tblFMetas" ref="A4:H9" headerRowCount="1">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblFMetas" displayName="tblFMetas" ref="A4:H9" headerRowCount="1">
   <autoFilter ref="A4:H9"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Meta"/>
@@ -519,8 +583,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblFCompromisos" displayName="tblFCompromisos" ref="A4:E9" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblFCompromisos" displayName="tblFCompromisos" ref="A4:E9" headerRowCount="1">
   <autoFilter ref="A4:E9"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Compromiso"/>
@@ -533,8 +597,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblFAvances" displayName="tblFAvances" ref="A4:D9" headerRowCount="1">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblFAvances" displayName="tblFAvances" ref="A4:D9" headerRowCount="1">
   <autoFilter ref="A4:D9"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Fecha"/>
@@ -546,36 +610,12 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblFAcepto" displayName="tblFAcepto" ref="A4:B5" headerRowCount="1">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblFAcepto" displayName="tblFAcepto" ref="A4:B5" headerRowCount="1">
   <autoFilter ref="A4:B5"/>
   <tableColumns count="2">
     <tableColumn id="1" name="De acuerdo"/>
     <tableColumn id="2" name="Fecha"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblFSugeridas" displayName="tblFSugeridas" ref="A4:D11" headerRowCount="1">
-  <autoFilter ref="A4:D11"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Meta"/>
-    <tableColumn id="2" name="M · Medible"/>
-    <tableColumn id="3" name="Plazo (días)"/>
-    <tableColumn id="4" name="Área"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblFInfo" displayName="tblFInfo" ref="A1:B5" headerRowCount="1">
-  <autoFilter ref="A1:B5"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Clave"/>
-    <tableColumn id="2" name="Valor"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1132,6 +1172,16 @@
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
+          <t>Mi plan</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Mis lecturas</t>
+        </is>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
           <t>Ideas de metas</t>
         </is>
       </c>
@@ -1192,13 +1242,823 @@
     <hyperlink ref="I16" location="'Mis compromisos'!A1" display="Mis compromisos"/>
     <hyperlink ref="K16" location="'Mis avances'!A1" display="Mis avances"/>
     <hyperlink ref="L16" location="'Acuerdo'!A1" display="Acuerdo"/>
-    <hyperlink ref="E17" location="'Ideas de metas'!A1" display="Ideas de metas"/>
+    <hyperlink ref="E17" location="'Mi plan'!A1" display="Mi plan"/>
+    <hyperlink ref="F17" location="'Mis lecturas'!A1" display="Mis lecturas"/>
+    <hyperlink ref="H17" location="'Ideas de metas'!A1" display="Ideas de metas"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0060A5FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PARA CONSULTAR   ·   ← Mi cabina</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Ideas para tus metas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Para inspirarte: adáptalas y escríbelas en «Mis metas» con tus propios números.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>M · Medible</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Plazo (días)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Área</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Proyecto ancla: construir un asistente o agente que resuelva un flujo completo de mi área</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Demo funcionando en la sesión 6, usada por al menos 2 compañeros y con horas ahorradas medidas</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>120</v>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Agentes y automatización</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Medir la calidad de mi mejor GPT con 20 casos de prueba</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Tasa de acierto medida antes y después de mejorarlo (meta: +20 puntos)</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Evaluación y calidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Comparar ChatGPT, Claude y Gemini en mis 5 tareas más importantes</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Tabla con ganador por tarea y por qué, y un cambio de herramienta en al menos una tarea</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Criterio multi-modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Armar un GPT o Project con el conocimiento de mi área que responda citando la fuente</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Responde bien 8 de 10 preguntas reales y siempre cita la fuente</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>45</v>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Contexto y conocimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Presentar a mi jefe un caso de negocio de IA con el ROI medido</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Presentado con números reales y con una decisión: escalar, ajustar o parar</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>90</v>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Impacto de negocio</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Analizar con IA y código un archivo real y sacar 3 hallazgos verificados</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>3 hallazgos verificados contra la fuente y una gráfica que se entienda sola</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Datos y análisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Llevar la IA a mi equipo: taller de 30 minutos y reglas de uso</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Taller dado, reglas de una página aprobadas y 3 compañeros usándolo</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>60</v>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Adopción y riesgo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Mi cabina'!A1" display="PARA CONSULTAR   ·   ← Mi cabina"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>archivo</t>
+        </is>
+      </c>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>mentoria-fernando</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="B3" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>mentee</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Fernando</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Valeria</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0060A5FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PARA CONSULTAR   ·   ← Mi cabina</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Mi plan de trabajo, sesión por sesión</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Lo que te toca en cada sesión y lo que se entrega. Tú llevas el volante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Sesión</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Enfoque</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Lo que me toca</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Conocerse, acuerdo, metas y elegir el proyecto ancla</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Llenar su Radar IA y su preparación en su Excel.
+Traer su mejor GPT y su peor alucinación.
+Proponer un problema real de su área como proyecto ancla.</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Proyecto ancla elegido y Radar IA de línea base</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="64" customHeight="1">
+      <c r="A6" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Medir el punto de partida y diseñar la solución</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Medir cuánto tarda y cuánto falla hoy el proceso.
+Diseñar su solución en una página.</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Cuánto tarda y cuánto falla hoy el proceso; diseño en una página</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="64" customHeight="1">
+      <c r="A7" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Prototipo y check-in de mitad de ciclo</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Traer algo funcionando, aunque sea feo.
+Radar IA de mitad de ciclo.</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Algo funcionando, aunque sea feo; Radar IA de mitad de ciclo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Probar en serio: casos de prueba y comparar modelos</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Armar 20 casos de prueba con su respuesta correcta.
+Probarlos en 2 o 3 herramientas y sacar la tasa de acierto.</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>20 casos de prueba con su tasa de acierto y la mejor herramienta para cada paso</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Piloto con usuarios reales</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>Que dos compañeros lo usen una semana.
+Medir horas ahorradas y errores.</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Dos compañeros usándolo y horas ahorradas medidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="64" customHeight="1">
+      <c r="A10" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Demo day y red</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Presentar a su jefe o equipo con números.
+Radar IA final y qué sigue para su proyecto.</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Presentación a su jefe o equipo con números, 2 o 3 presentaciones con gente de la red de Valeria y Radar IA final</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Mi cabina'!A1" display="PARA CONSULTAR   ·   ← Mi cabina"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0060A5FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PARA CONSULTAR   ·   ← Mi cabina</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Mis lecturas, una por sesión</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Gratis y con liga directa: clic en la liga para abrirla o descargarla. Están en inglés: la página web se traduce con clic derecho → Traducir; un PDF lo puedes subir a la IA y pedirle un resumen en español.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Sesión</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Autor</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Por qué leerla</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>15 Times to use AI, and 5 Not to</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Ethan Mollick (One Useful Thing, 2024)</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="30" t="inlineStr">
+        <is>
+          <t>Criterio para saber cuándo sí conviene la IA y cuándo no. Ayuda a elegir bien el proyecto ancla.</t>
+        </is>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>https://www.oneusefulthing.org/p/15-times-to-use-ai-and-5-not-to</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Identifying and scaling AI use cases</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>OpenAI (2025)</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>Cómo encontrar y priorizar casos de uso en tu área. Sirve para medir el punto de partida y diseñar la solución.</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="inlineStr">
+        <is>
+          <t>https://cdn.openai.com/business-guides-and-resources/identifying-and-scaling-ai-use-cases.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>A practical guide to building agents</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>OpenAI (2025)</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>Modelo, herramientas e instrucciones: lo básico para armar el prototipo de un agente.</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>https://cdn.openai.com/business-guides-and-resources/a-practical-guide-to-building-agents.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Building effective agents</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Anthropic (2024)</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>Complemento: empezar con flujos simples antes que agentes complejos.</t>
+        </is>
+      </c>
+      <c r="G8" s="32" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/engineering/building-effective-agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Your AI Product Needs Evals</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>Hamel Husain (2024)</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>Cómo armar casos de prueba y medir la tasa de acierto: justo sus 20 casos.</t>
+        </is>
+      </c>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>https://hamel.dev/blog/posts/evals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>People + AI Guidebook</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Google PAIR</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>Cómo diseñar algo con IA que la gente sí use: confianza, errores y retroalimentación. Para el piloto con usuarios.</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>https://pair.withgoogle.com/guidebook/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>AI in the Enterprise</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>OpenAI (2025)</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Siete lecciones de empresas que ya escalaron la IA. Ideas para presentar su caso con números en el demo day.</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>https://cdn.openai.com/business-guides-and-resources/ai-in-the-enterprise.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Mi cabina'!A1" display="PARA CONSULTAR   ·   ← Mi cabina"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId7"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -1246,60 +2106,60 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Llenar mi Radar IA con la escala nueva: siete áreas, del 1 al 5.</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Tener listo para mostrar mi mejor GPT, prompt o automatización (3 minutos).</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Traer mi peor alucinación: cuándo me engañó la IA y cómo lo detecté.</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Traer un problema real de mi área que cueste horas o dinero: candidato a proyecto ancla.</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Anotar qué me dio la liga de IA y qué me faltó.</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -1326,7 +2186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -1397,14 +2257,14 @@
           <t>Criterio multi-modelo</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Elegir ChatGPT, Claude, Gemini o Copilot según la tarea, con pruebas y no por costumbre</t>
         </is>
       </c>
-      <c r="C5" s="30" t="n"/>
-      <c r="D5" s="30" t="n"/>
-      <c r="E5" s="30" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="29" t="n"/>
+      <c r="E5" s="29" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -1412,14 +2272,14 @@
           <t>Contexto y conocimiento</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>GPTs, Projects e instrucciones con documentos propios: que la IA conozca tu trabajo</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n"/>
-      <c r="D6" s="30" t="n"/>
-      <c r="E6" s="30" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="29" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
@@ -1427,14 +2287,14 @@
           <t>Agentes y automatización</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Flujos de punta a punta con herramientas conectadas: acciones, conectores, Power Automate, API</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n"/>
-      <c r="D7" s="30" t="n"/>
-      <c r="E7" s="30" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
@@ -1442,14 +2302,14 @@
           <t>Evaluación y calidad</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Saber si la IA lo hace bien: casos de prueba, rúbricas, tasa de error y fuentes verificadas</t>
         </is>
       </c>
-      <c r="C8" s="30" t="n"/>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="30" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
@@ -1457,14 +2317,14 @@
           <t>Datos y análisis</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Análisis con código (Python, Excel) y hallazgos verificados contra la fuente</t>
         </is>
       </c>
-      <c r="C9" s="30" t="n"/>
-      <c r="D9" s="30" t="n"/>
-      <c r="E9" s="30" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="29" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
@@ -1472,14 +2332,14 @@
           <t>Impacto de negocio</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
         <is>
           <t>Casos con ROI medido, antes y después, y una historia que convenza a tu jefe</t>
         </is>
       </c>
-      <c r="C10" s="30" t="n"/>
-      <c r="D10" s="30" t="n"/>
-      <c r="E10" s="30" t="n"/>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
@@ -1487,17 +2347,17 @@
           <t>Adopción y riesgo</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Llevar la IA a tu equipo con reglas claras: datos sensibles, sesgos y uso responsable</t>
         </is>
       </c>
-      <c r="C11" s="30" t="n"/>
-      <c r="D11" s="30" t="n"/>
-      <c r="E11" s="30" t="n"/>
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>La escala</t>
         </is>
@@ -1521,77 +2381,77 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>Lo conozco</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Sé qué es y para qué sirve, pero no lo uso.</t>
         </is>
       </c>
-      <c r="C16" s="30" t="n">
+      <c r="C16" s="29" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>Lo uso en el chat</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Lo uso de vez en cuando, caso por caso.</t>
         </is>
       </c>
-      <c r="C17" s="30" t="n">
+      <c r="C17" s="29" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Lo uso con método</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>Es parte de mi semana y tengo una forma repetible de hacerlo.</t>
         </is>
       </c>
-      <c r="C18" s="30" t="n">
+      <c r="C18" s="29" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Construyo para otros</t>
         </is>
       </c>
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>Hice algo que otras personas usan sin mí.</t>
         </is>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="29" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Lo mido y lo escalo</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>Tengo números del impacto y lo enseño o lo llevo a más áreas.</t>
         </is>
       </c>
-      <c r="C20" s="30" t="n">
+      <c r="C20" s="29" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1613,7 +2473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -1697,54 +2557,54 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="29" t="n"/>
-      <c r="B5" s="29" t="n"/>
-      <c r="C5" s="29" t="n"/>
-      <c r="D5" s="29" t="n"/>
-      <c r="E5" s="29" t="n"/>
-      <c r="F5" s="33" t="n"/>
-      <c r="G5" s="29" t="n"/>
-      <c r="H5" s="34" t="n"/>
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" s="30" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="30" t="n"/>
+      <c r="F5" s="34" t="n"/>
+      <c r="G5" s="30" t="n"/>
+      <c r="H5" s="35" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="29" t="n"/>
-      <c r="B6" s="29" t="n"/>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
-      <c r="E6" s="29" t="n"/>
-      <c r="F6" s="33" t="n"/>
-      <c r="G6" s="29" t="n"/>
-      <c r="H6" s="34" t="n"/>
+      <c r="A6" s="30" t="n"/>
+      <c r="B6" s="30" t="n"/>
+      <c r="C6" s="30" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="30" t="n"/>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="30" t="n"/>
+      <c r="H6" s="35" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="29" t="n"/>
-      <c r="B7" s="29" t="n"/>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="29" t="n"/>
-      <c r="E7" s="29" t="n"/>
-      <c r="F7" s="33" t="n"/>
-      <c r="G7" s="29" t="n"/>
-      <c r="H7" s="34" t="n"/>
+      <c r="A7" s="30" t="n"/>
+      <c r="B7" s="30" t="n"/>
+      <c r="C7" s="30" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="30" t="n"/>
+      <c r="F7" s="34" t="n"/>
+      <c r="G7" s="30" t="n"/>
+      <c r="H7" s="35" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="29" t="n"/>
-      <c r="B8" s="29" t="n"/>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="29" t="n"/>
-      <c r="F8" s="33" t="n"/>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="34" t="n"/>
+      <c r="A8" s="30" t="n"/>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="34" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="35" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
-      <c r="E9" s="29" t="n"/>
-      <c r="F9" s="33" t="n"/>
-      <c r="G9" s="29" t="n"/>
-      <c r="H9" s="34" t="n"/>
+      <c r="A9" s="30" t="n"/>
+      <c r="B9" s="30" t="n"/>
+      <c r="C9" s="30" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="30" t="n"/>
+      <c r="F9" s="34" t="n"/>
+      <c r="G9" s="30" t="n"/>
+      <c r="H9" s="35" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1770,7 +2630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -1836,39 +2696,39 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="n"/>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="30" t="n"/>
-      <c r="D5" s="29" t="n"/>
-      <c r="E5" s="30" t="n"/>
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="34" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="29" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="n"/>
-      <c r="B6" s="33" t="n"/>
-      <c r="C6" s="30" t="n"/>
-      <c r="D6" s="29" t="n"/>
-      <c r="E6" s="30" t="n"/>
+      <c r="A6" s="30" t="n"/>
+      <c r="B6" s="34" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="29" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="n"/>
-      <c r="B7" s="33" t="n"/>
-      <c r="C7" s="30" t="n"/>
-      <c r="D7" s="29" t="n"/>
-      <c r="E7" s="30" t="n"/>
+      <c r="A7" s="30" t="n"/>
+      <c r="B7" s="34" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="29" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="n"/>
-      <c r="B8" s="33" t="n"/>
-      <c r="C8" s="30" t="n"/>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="30" t="n"/>
+      <c r="A8" s="30" t="n"/>
+      <c r="B8" s="34" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="29" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="33" t="n"/>
-      <c r="C9" s="30" t="n"/>
-      <c r="D9" s="29" t="n"/>
-      <c r="E9" s="30" t="n"/>
+      <c r="A9" s="30" t="n"/>
+      <c r="B9" s="34" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="29" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A5:E300">
@@ -1894,7 +2754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -1954,34 +2814,34 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="33" t="n"/>
-      <c r="B5" s="29" t="n"/>
-      <c r="C5" s="29" t="n"/>
-      <c r="D5" s="29" t="n"/>
+      <c r="A5" s="34" t="n"/>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" s="30" t="n"/>
+      <c r="D5" s="30" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="33" t="n"/>
-      <c r="B6" s="29" t="n"/>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
+      <c r="A6" s="34" t="n"/>
+      <c r="B6" s="30" t="n"/>
+      <c r="C6" s="30" t="n"/>
+      <c r="D6" s="30" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="29" t="n"/>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="29" t="n"/>
+      <c r="A7" s="34" t="n"/>
+      <c r="B7" s="30" t="n"/>
+      <c r="C7" s="30" t="n"/>
+      <c r="D7" s="30" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="29" t="n"/>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
+      <c r="A8" s="34" t="n"/>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
+      <c r="A9" s="34" t="n"/>
+      <c r="B9" s="30" t="n"/>
+      <c r="C9" s="30" t="n"/>
+      <c r="D9" s="30" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2000,7 +2860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -2048,8 +2908,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n"/>
-      <c r="B5" s="33" t="n"/>
+      <c r="A5" s="29" t="n"/>
+      <c r="B5" s="34" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A5:B5">
@@ -2073,289 +2933,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="0060A5FA"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PARA CONSULTAR   ·   ← Mi cabina</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Ideas para tus metas</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>Para inspirarte: adáptalas y escríbelas en «Mis metas» con tus propios números.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>M · Medible</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>Plazo (días)</t>
-        </is>
-      </c>
-      <c r="D4" s="28" t="inlineStr">
-        <is>
-          <t>Área</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>Proyecto ancla: construir un asistente o agente que resuelva un flujo completo de mi área</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>Demo funcionando en la sesión 6, usada por al menos 2 compañeros y con horas ahorradas medidas</t>
-        </is>
-      </c>
-      <c r="C5" s="30" t="n">
-        <v>120</v>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
-        <is>
-          <t>Agentes y automatización</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Medir la calidad de mi mejor GPT con 20 casos de prueba</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="inlineStr">
-        <is>
-          <t>Tasa de acierto medida antes y después de mejorarlo (meta: +20 puntos)</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="n">
-        <v>45</v>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>Evaluación y calidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Comparar ChatGPT, Claude y Gemini en mis 5 tareas más importantes</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>Tabla con ganador por tarea y por qué, y un cambio de herramienta en al menos una tarea</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="n">
-        <v>30</v>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>Criterio multi-modelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Armar un GPT o Project con el conocimiento de mi área que responda citando la fuente</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>Responde bien 8 de 10 preguntas reales y siempre cita la fuente</t>
-        </is>
-      </c>
-      <c r="C8" s="30" t="n">
-        <v>45</v>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>Contexto y conocimiento</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Presentar a mi jefe un caso de negocio de IA con el ROI medido</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>Presentado con números reales y con una decisión: escalar, ajustar o parar</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="n">
-        <v>90</v>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>Impacto de negocio</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Analizar con IA y código un archivo real y sacar 3 hallazgos verificados</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>3 hallazgos verificados contra la fuente y una gráfica que se entienda sola</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="n">
-        <v>45</v>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>Datos y análisis</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Llevar la IA a mi equipo: taller de 30 minutos y reglas de uso</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Taller dado, reglas de una página aprobadas y 3 compañeros usándolo</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="n">
-        <v>60</v>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>Adopción y riesgo</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Mi cabina'!A1" display="PARA CONSULTAR   ·   ← Mi cabina"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
-        <is>
-          <t>Clave</t>
-        </is>
-      </c>
-      <c r="B1" s="28" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="29" t="inlineStr">
-        <is>
-          <t>archivo</t>
-        </is>
-      </c>
-      <c r="B2" s="29" t="inlineStr">
-        <is>
-          <t>mentoria-fernando</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="29" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="B3" s="29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>mentee</t>
-        </is>
-      </c>
-      <c r="B4" s="29" t="inlineStr">
-        <is>
-          <t>Fernando</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>mentor</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>Valeria</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>